<commit_message>
Complete dashboard APIs and add call follow-up conversion stats
</commit_message>
<xml_diff>
--- a/excel_data/leads.xlsx
+++ b/excel_data/leads.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -499,6 +499,106 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>raj rajak</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>raj79@gmail.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1256374658</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>converted</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>raj rajak</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>raj79@gmail.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1256374658</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>converted</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>raj rajak</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>raj79@gmail.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1256374658</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>converted</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>raja rajak</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>raj79@gmail.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1256374658</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>